<commit_message>
docs(b4.3): record Phase B WBS completion
</commit_message>
<xml_diff>
--- a/ESP32_S3_SQD_Project_WBS.xlsx
+++ b/ESP32_S3_SQD_Project_WBS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f91d42a59b2d5e5/SQD/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive\SQD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{C84441A9-493A-415C-B430-AB0EFCA297E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7038D520-20FD-4BCA-A22B-CE50EC350255}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97F445B2-9959-4A2B-953A-FF2A2BEAA89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14085" yWindow="-16200" windowWidth="29010" windowHeight="15585" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-14730" yWindow="-16320" windowWidth="57840" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -3831,7 +3831,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.37037037037037041</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4318,14 +4318,14 @@
       </c>
       <c r="E5" s="12">
         <f>Control!B11</f>
-        <v>0.11553133514986372</v>
+        <v>0.17111716621253398</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>6</v>
       </c>
       <c r="H5" s="12">
         <f>Control!B12</f>
-        <v>0.10463215258855582</v>
+        <v>0.16021798365122608</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="30" customHeight="1"/>
@@ -4342,7 +4342,7 @@
       </c>
       <c r="E7" s="11">
         <f>Control!B14</f>
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>9</v>
@@ -4447,11 +4447,11 @@
       </c>
       <c r="F13" s="6">
         <f>IFERROR(SUMIF(WBS!$B$5:$B$137,A13,WBS!$T$5:$T$137)/SUMIF(WBS!$B$5:$B$137,A13,WBS!$R$5:$R$137),0)</f>
-        <v>0.37037037037037041</v>
+        <v>1</v>
       </c>
       <c r="G13" s="6">
         <f t="shared" si="0"/>
-        <v>0.37037037037037041</v>
+        <v>1</v>
       </c>
       <c r="H13" s="4">
         <f>COUNTIF(WBS!$B$5:$B$137,A13)</f>
@@ -4459,7 +4459,7 @@
       </c>
       <c r="I13" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A13,WBS!$U$5:$U$137,"Complete")</f>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="J13" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A13,WBS!$U$5:$U$137,"Late")</f>
@@ -4947,7 +4947,7 @@
       </c>
       <c r="B11" s="6">
         <f>SUM(WBS!T5:T137)</f>
-        <v>0.11553133514986372</v>
+        <v>0.17111716621253398</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>69</v>
@@ -4962,7 +4962,7 @@
       </c>
       <c r="B12" s="6">
         <f>B11-B10</f>
-        <v>0.10463215258855582</v>
+        <v>0.16021798365122608</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>70</v>
@@ -4992,7 +4992,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF(WBS!U5:U137,"Complete")</f>
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>72</v>
@@ -6386,7 +6386,7 @@
         <v>0</v>
       </c>
       <c r="Q20" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R20" s="14">
         <f t="shared" si="0"/>
@@ -6398,11 +6398,11 @@
       </c>
       <c r="T20" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.4495912806539499E-3</v>
       </c>
       <c r="U20" t="str">
         <f>IF(Q20&gt;=1,"Complete",IF(Q20&gt;0,"In Progress",IF(Control!$B$7&lt;H20,"Not Started",IF(Control!$B$7&gt;I20,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V20" s="15">
         <v>46272</v>
@@ -6459,7 +6459,7 @@
         <v>0</v>
       </c>
       <c r="Q21" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R21" s="14">
         <f t="shared" si="0"/>
@@ -6471,11 +6471,11 @@
       </c>
       <c r="T21" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.08991825613079E-2</v>
       </c>
       <c r="U21" t="str">
         <f>IF(Q21&gt;=1,"Complete",IF(Q21&gt;0,"In Progress",IF(Control!$B$7&lt;H21,"Not Started",IF(Control!$B$7&gt;I21,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V21" s="15">
         <v>46272</v>
@@ -6532,7 +6532,7 @@
         <v>0</v>
       </c>
       <c r="Q22" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R22" s="14">
         <f t="shared" si="0"/>
@@ -6544,11 +6544,11 @@
       </c>
       <c r="T22" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.08991825613079E-2</v>
       </c>
       <c r="U22" t="str">
         <f>IF(Q22&gt;=1,"Complete",IF(Q22&gt;0,"In Progress",IF(Control!$B$7&lt;H22,"Not Started",IF(Control!$B$7&gt;I22,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V22" s="15">
         <v>46279</v>
@@ -6605,7 +6605,7 @@
         <v>0</v>
       </c>
       <c r="Q23" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R23" s="14">
         <f t="shared" si="0"/>
@@ -6617,11 +6617,11 @@
       </c>
       <c r="T23" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.4495912806539499E-3</v>
       </c>
       <c r="U23" t="str">
         <f>IF(Q23&gt;=1,"Complete",IF(Q23&gt;0,"In Progress",IF(Control!$B$7&lt;H23,"Not Started",IF(Control!$B$7&gt;I23,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V23" s="15">
         <v>46286</v>
@@ -6678,7 +6678,7 @@
         <v>0</v>
       </c>
       <c r="Q24" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R24" s="14">
         <f t="shared" si="0"/>
@@ -6690,11 +6690,11 @@
       </c>
       <c r="T24" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.08991825613079E-2</v>
       </c>
       <c r="U24" t="str">
         <f>IF(Q24&gt;=1,"Complete",IF(Q24&gt;0,"In Progress",IF(Control!$B$7&lt;H24,"Not Started",IF(Control!$B$7&gt;I24,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V24" s="15">
         <v>46286</v>
@@ -6751,7 +6751,7 @@
         <v>0</v>
       </c>
       <c r="Q25" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R25" s="14">
         <f t="shared" si="0"/>
@@ -6763,11 +6763,11 @@
       </c>
       <c r="T25" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.4495912806539499E-3</v>
       </c>
       <c r="U25" t="str">
         <f>IF(Q25&gt;=1,"Complete",IF(Q25&gt;0,"In Progress",IF(Control!$B$7&lt;H25,"Not Started",IF(Control!$B$7&gt;I25,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V25" s="15">
         <v>46293</v>
@@ -6827,7 +6827,7 @@
         <v>0</v>
       </c>
       <c r="Q26" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R26" s="14">
         <f t="shared" si="0"/>
@@ -6839,11 +6839,11 @@
       </c>
       <c r="T26" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>6.5395095367847397E-3</v>
       </c>
       <c r="U26" t="str">
         <f>IF(Q26&gt;=1,"Complete",IF(Q26&gt;0,"In Progress",IF(Control!$B$7&lt;H26,"Not Started",IF(Control!$B$7&gt;I26,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V26" s="15">
         <v>46293</v>
@@ -15314,22 +15314,22 @@
       </c>
       <c r="H8" s="6">
         <f>IFERROR(SUMIF(WBS!$D$5:$D$137,A8,WBS!$T$5:$T$137)/SUMIF(WBS!$D$5:$D$137,A8,WBS!$R$5:$R$137),0)</f>
-        <v>0.66666666666666663</v>
+        <v>1</v>
       </c>
       <c r="I8" s="6">
         <f t="shared" si="0"/>
-        <v>0.66666666666666663</v>
+        <v>1</v>
       </c>
       <c r="J8" s="4">
         <v>3</v>
       </c>
       <c r="K8" s="4">
         <f>COUNTIFS(WBS!$D$5:$D$137,A8,WBS!$U$5:$U$137,"Complete")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L8" s="4" t="str">
         <f>IF(H8&gt;=1,"Complete",IF(H8&gt;0,"In Progress",IF(Control!$B$7&lt;D8,"Not Started",IF(Control!$B$7&gt;E8,"Late","Ready"))))</f>
-        <v>In Progress</v>
+        <v>Complete</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -15357,22 +15357,22 @@
       </c>
       <c r="H9" s="6">
         <f>IFERROR(SUMIF(WBS!$D$5:$D$137,A9,WBS!$T$5:$T$137)/SUMIF(WBS!$D$5:$D$137,A9,WBS!$R$5:$R$137),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" s="4">
         <v>3</v>
       </c>
       <c r="K9" s="4">
         <f>COUNTIFS(WBS!$D$5:$D$137,A9,WBS!$U$5:$U$137,"Complete")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L9" s="4" t="str">
         <f>IF(H9&gt;=1,"Complete",IF(H9&gt;0,"In Progress",IF(Control!$B$7&lt;D9,"Not Started",IF(Control!$B$7&gt;E9,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -15400,22 +15400,22 @@
       </c>
       <c r="H10" s="6">
         <f>IFERROR(SUMIF(WBS!$D$5:$D$137,A10,WBS!$T$5:$T$137)/SUMIF(WBS!$D$5:$D$137,A10,WBS!$R$5:$R$137),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" s="4">
         <v>3</v>
       </c>
       <c r="K10" s="4">
         <f>COUNTIFS(WBS!$D$5:$D$137,A10,WBS!$U$5:$U$137,"Complete")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L10" s="4" t="str">
         <f>IF(H10&gt;=1,"Complete",IF(H10&gt;0,"In Progress",IF(Control!$B$7&lt;D10,"Not Started",IF(Control!$B$7&gt;E10,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -16969,7 +16969,7 @@
       </c>
       <c r="I4" s="6">
         <f>IF(A4=Control!$B$7,Control!$B$11,"")</f>
-        <v>0.11553133514986372</v>
+        <v>0.17111716621253398</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="42.75">

</xml_diff>

<commit_message>
docs(b4.3): record Phase B WBS completion (#18)
</commit_message>
<xml_diff>
--- a/ESP32_S3_SQD_Project_WBS.xlsx
+++ b/ESP32_S3_SQD_Project_WBS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f91d42a59b2d5e5/SQD/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive\SQD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{C84441A9-493A-415C-B430-AB0EFCA297E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7038D520-20FD-4BCA-A22B-CE50EC350255}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97F445B2-9959-4A2B-953A-FF2A2BEAA89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14085" yWindow="-16200" windowWidth="29010" windowHeight="15585" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-14730" yWindow="-16320" windowWidth="57840" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -3831,7 +3831,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.37037037037037041</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4318,14 +4318,14 @@
       </c>
       <c r="E5" s="12">
         <f>Control!B11</f>
-        <v>0.11553133514986372</v>
+        <v>0.17111716621253398</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>6</v>
       </c>
       <c r="H5" s="12">
         <f>Control!B12</f>
-        <v>0.10463215258855582</v>
+        <v>0.16021798365122608</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="30" customHeight="1"/>
@@ -4342,7 +4342,7 @@
       </c>
       <c r="E7" s="11">
         <f>Control!B14</f>
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>9</v>
@@ -4447,11 +4447,11 @@
       </c>
       <c r="F13" s="6">
         <f>IFERROR(SUMIF(WBS!$B$5:$B$137,A13,WBS!$T$5:$T$137)/SUMIF(WBS!$B$5:$B$137,A13,WBS!$R$5:$R$137),0)</f>
-        <v>0.37037037037037041</v>
+        <v>1</v>
       </c>
       <c r="G13" s="6">
         <f t="shared" si="0"/>
-        <v>0.37037037037037041</v>
+        <v>1</v>
       </c>
       <c r="H13" s="4">
         <f>COUNTIF(WBS!$B$5:$B$137,A13)</f>
@@ -4459,7 +4459,7 @@
       </c>
       <c r="I13" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A13,WBS!$U$5:$U$137,"Complete")</f>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="J13" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A13,WBS!$U$5:$U$137,"Late")</f>
@@ -4947,7 +4947,7 @@
       </c>
       <c r="B11" s="6">
         <f>SUM(WBS!T5:T137)</f>
-        <v>0.11553133514986372</v>
+        <v>0.17111716621253398</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>69</v>
@@ -4962,7 +4962,7 @@
       </c>
       <c r="B12" s="6">
         <f>B11-B10</f>
-        <v>0.10463215258855582</v>
+        <v>0.16021798365122608</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>70</v>
@@ -4992,7 +4992,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF(WBS!U5:U137,"Complete")</f>
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>72</v>
@@ -6386,7 +6386,7 @@
         <v>0</v>
       </c>
       <c r="Q20" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R20" s="14">
         <f t="shared" si="0"/>
@@ -6398,11 +6398,11 @@
       </c>
       <c r="T20" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.4495912806539499E-3</v>
       </c>
       <c r="U20" t="str">
         <f>IF(Q20&gt;=1,"Complete",IF(Q20&gt;0,"In Progress",IF(Control!$B$7&lt;H20,"Not Started",IF(Control!$B$7&gt;I20,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V20" s="15">
         <v>46272</v>
@@ -6459,7 +6459,7 @@
         <v>0</v>
       </c>
       <c r="Q21" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R21" s="14">
         <f t="shared" si="0"/>
@@ -6471,11 +6471,11 @@
       </c>
       <c r="T21" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.08991825613079E-2</v>
       </c>
       <c r="U21" t="str">
         <f>IF(Q21&gt;=1,"Complete",IF(Q21&gt;0,"In Progress",IF(Control!$B$7&lt;H21,"Not Started",IF(Control!$B$7&gt;I21,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V21" s="15">
         <v>46272</v>
@@ -6532,7 +6532,7 @@
         <v>0</v>
       </c>
       <c r="Q22" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R22" s="14">
         <f t="shared" si="0"/>
@@ -6544,11 +6544,11 @@
       </c>
       <c r="T22" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.08991825613079E-2</v>
       </c>
       <c r="U22" t="str">
         <f>IF(Q22&gt;=1,"Complete",IF(Q22&gt;0,"In Progress",IF(Control!$B$7&lt;H22,"Not Started",IF(Control!$B$7&gt;I22,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V22" s="15">
         <v>46279</v>
@@ -6605,7 +6605,7 @@
         <v>0</v>
       </c>
       <c r="Q23" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R23" s="14">
         <f t="shared" si="0"/>
@@ -6617,11 +6617,11 @@
       </c>
       <c r="T23" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.4495912806539499E-3</v>
       </c>
       <c r="U23" t="str">
         <f>IF(Q23&gt;=1,"Complete",IF(Q23&gt;0,"In Progress",IF(Control!$B$7&lt;H23,"Not Started",IF(Control!$B$7&gt;I23,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V23" s="15">
         <v>46286</v>
@@ -6678,7 +6678,7 @@
         <v>0</v>
       </c>
       <c r="Q24" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R24" s="14">
         <f t="shared" si="0"/>
@@ -6690,11 +6690,11 @@
       </c>
       <c r="T24" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.08991825613079E-2</v>
       </c>
       <c r="U24" t="str">
         <f>IF(Q24&gt;=1,"Complete",IF(Q24&gt;0,"In Progress",IF(Control!$B$7&lt;H24,"Not Started",IF(Control!$B$7&gt;I24,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V24" s="15">
         <v>46286</v>
@@ -6751,7 +6751,7 @@
         <v>0</v>
       </c>
       <c r="Q25" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R25" s="14">
         <f t="shared" si="0"/>
@@ -6763,11 +6763,11 @@
       </c>
       <c r="T25" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.4495912806539499E-3</v>
       </c>
       <c r="U25" t="str">
         <f>IF(Q25&gt;=1,"Complete",IF(Q25&gt;0,"In Progress",IF(Control!$B$7&lt;H25,"Not Started",IF(Control!$B$7&gt;I25,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V25" s="15">
         <v>46293</v>
@@ -6827,7 +6827,7 @@
         <v>0</v>
       </c>
       <c r="Q26" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R26" s="14">
         <f t="shared" si="0"/>
@@ -6839,11 +6839,11 @@
       </c>
       <c r="T26" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>6.5395095367847397E-3</v>
       </c>
       <c r="U26" t="str">
         <f>IF(Q26&gt;=1,"Complete",IF(Q26&gt;0,"In Progress",IF(Control!$B$7&lt;H26,"Not Started",IF(Control!$B$7&gt;I26,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V26" s="15">
         <v>46293</v>
@@ -15314,22 +15314,22 @@
       </c>
       <c r="H8" s="6">
         <f>IFERROR(SUMIF(WBS!$D$5:$D$137,A8,WBS!$T$5:$T$137)/SUMIF(WBS!$D$5:$D$137,A8,WBS!$R$5:$R$137),0)</f>
-        <v>0.66666666666666663</v>
+        <v>1</v>
       </c>
       <c r="I8" s="6">
         <f t="shared" si="0"/>
-        <v>0.66666666666666663</v>
+        <v>1</v>
       </c>
       <c r="J8" s="4">
         <v>3</v>
       </c>
       <c r="K8" s="4">
         <f>COUNTIFS(WBS!$D$5:$D$137,A8,WBS!$U$5:$U$137,"Complete")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L8" s="4" t="str">
         <f>IF(H8&gt;=1,"Complete",IF(H8&gt;0,"In Progress",IF(Control!$B$7&lt;D8,"Not Started",IF(Control!$B$7&gt;E8,"Late","Ready"))))</f>
-        <v>In Progress</v>
+        <v>Complete</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -15357,22 +15357,22 @@
       </c>
       <c r="H9" s="6">
         <f>IFERROR(SUMIF(WBS!$D$5:$D$137,A9,WBS!$T$5:$T$137)/SUMIF(WBS!$D$5:$D$137,A9,WBS!$R$5:$R$137),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" s="4">
         <v>3</v>
       </c>
       <c r="K9" s="4">
         <f>COUNTIFS(WBS!$D$5:$D$137,A9,WBS!$U$5:$U$137,"Complete")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L9" s="4" t="str">
         <f>IF(H9&gt;=1,"Complete",IF(H9&gt;0,"In Progress",IF(Control!$B$7&lt;D9,"Not Started",IF(Control!$B$7&gt;E9,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -15400,22 +15400,22 @@
       </c>
       <c r="H10" s="6">
         <f>IFERROR(SUMIF(WBS!$D$5:$D$137,A10,WBS!$T$5:$T$137)/SUMIF(WBS!$D$5:$D$137,A10,WBS!$R$5:$R$137),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I10" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" s="4">
         <v>3</v>
       </c>
       <c r="K10" s="4">
         <f>COUNTIFS(WBS!$D$5:$D$137,A10,WBS!$U$5:$U$137,"Complete")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L10" s="4" t="str">
         <f>IF(H10&gt;=1,"Complete",IF(H10&gt;0,"In Progress",IF(Control!$B$7&lt;D10,"Not Started",IF(Control!$B$7&gt;E10,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -16969,7 +16969,7 @@
       </c>
       <c r="I4" s="6">
         <f>IF(A4=Control!$B$7,Control!$B$11,"")</f>
-        <v>0.11553133514986372</v>
+        <v>0.17111716621253398</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="42.75">

</xml_diff>

<commit_message>
docs(c1.1): record architecture acceptance
Mark the C1.1 architecture as accepted and record PR, merged-main and CI evidence.

Update the C1.1 WBS row to 100 percent completion with acceptance traceability.
</commit_message>
<xml_diff>
--- a/ESP32_S3_SQD_Project_WBS.xlsx
+++ b/ESP32_S3_SQD_Project_WBS.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive\SQD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f91d42a59b2d5e5/SQD_WBS_Backups/B4.3_WBS_Recovery_20260726_091129/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97F445B2-9959-4A2B-953A-FF2A2BEAA89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{97F445B2-9959-4A2B-953A-FF2A2BEAA89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC2B6BFE-A532-4185-87E4-86725BF234C3}"/>
   <bookViews>
     <workbookView xWindow="-14730" yWindow="-16320" windowWidth="57840" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1973" uniqueCount="1048">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1974" uniqueCount="1049">
   <si>
     <t>ESP32-S3 Solo Program Dashboard</t>
   </si>
@@ -3319,6 +3319,9 @@
   </si>
   <si>
     <t>Parthasarathy CP</t>
+  </si>
+  <si>
+    <t>Architecture: docs/phase-c/C1.1_System_Architecture.md | PR: https://github.com/CPParthasarathy/SQD/pull/19 | Main: a56bb119c16f1f61adc0c9ab7c848496d6a2b52a | CI: https://github.com/CPParthasarathy/SQD/actions/runs/30207286673 (Quality contracts and all three ESP-IDF profiles green)</t>
   </si>
 </sst>
 </file>
@@ -3834,7 +3837,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>1.9920318725099608E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -4318,14 +4321,14 @@
       </c>
       <c r="E5" s="12">
         <f>Control!B11</f>
-        <v>0.17111716621253398</v>
+        <v>0.17656675749318793</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>6</v>
       </c>
       <c r="H5" s="12">
         <f>Control!B12</f>
-        <v>0.16021798365122608</v>
+        <v>0.16566757493188003</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="30" customHeight="1"/>
@@ -4342,7 +4345,7 @@
       </c>
       <c r="E7" s="11">
         <f>Control!B14</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>9</v>
@@ -4488,11 +4491,11 @@
       </c>
       <c r="F14" s="6">
         <f>IFERROR(SUMIF(WBS!$B$5:$B$137,A14,WBS!$T$5:$T$137)/SUMIF(WBS!$B$5:$B$137,A14,WBS!$R$5:$R$137),0)</f>
-        <v>0</v>
+        <v>1.9920318725099608E-2</v>
       </c>
       <c r="G14" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.9920318725099608E-2</v>
       </c>
       <c r="H14" s="4">
         <f>COUNTIF(WBS!$B$5:$B$137,A14)</f>
@@ -4500,7 +4503,7 @@
       </c>
       <c r="I14" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A14,WBS!$U$5:$U$137,"Complete")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A14,WBS!$U$5:$U$137,"Late")</f>
@@ -4947,7 +4950,7 @@
       </c>
       <c r="B11" s="6">
         <f>SUM(WBS!T5:T137)</f>
-        <v>0.17111716621253398</v>
+        <v>0.17656675749318793</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>69</v>
@@ -4962,7 +4965,7 @@
       </c>
       <c r="B12" s="6">
         <f>B11-B10</f>
-        <v>0.16021798365122608</v>
+        <v>0.16566757493188003</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>70</v>
@@ -4992,7 +4995,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF(WBS!U5:U137,"Complete")</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>72</v>
@@ -6119,7 +6122,7 @@
         <v>46271</v>
       </c>
     </row>
-    <row r="17" spans="1:23">
+    <row r="17" spans="1:24">
       <c r="A17" t="s">
         <v>165</v>
       </c>
@@ -6192,7 +6195,7 @@
         <v>46271</v>
       </c>
     </row>
-    <row r="18" spans="1:23">
+    <row r="18" spans="1:24">
       <c r="A18" t="s">
         <v>169</v>
       </c>
@@ -6265,7 +6268,7 @@
         <v>46271</v>
       </c>
     </row>
-    <row r="19" spans="1:23">
+    <row r="19" spans="1:24">
       <c r="A19" t="s">
         <v>175</v>
       </c>
@@ -6338,7 +6341,7 @@
         <v>46278</v>
       </c>
     </row>
-    <row r="20" spans="1:23">
+    <row r="20" spans="1:24">
       <c r="A20" t="s">
         <v>179</v>
       </c>
@@ -6411,7 +6414,7 @@
         <v>46278</v>
       </c>
     </row>
-    <row r="21" spans="1:23">
+    <row r="21" spans="1:24">
       <c r="A21" t="s">
         <v>183</v>
       </c>
@@ -6484,7 +6487,7 @@
         <v>46285</v>
       </c>
     </row>
-    <row r="22" spans="1:23">
+    <row r="22" spans="1:24">
       <c r="A22" t="s">
         <v>189</v>
       </c>
@@ -6557,7 +6560,7 @@
         <v>46292</v>
       </c>
     </row>
-    <row r="23" spans="1:23">
+    <row r="23" spans="1:24">
       <c r="A23" t="s">
         <v>193</v>
       </c>
@@ -6630,7 +6633,7 @@
         <v>46292</v>
       </c>
     </row>
-    <row r="24" spans="1:23">
+    <row r="24" spans="1:24">
       <c r="A24" t="s">
         <v>197</v>
       </c>
@@ -6703,7 +6706,7 @@
         <v>46299</v>
       </c>
     </row>
-    <row r="25" spans="1:23">
+    <row r="25" spans="1:24">
       <c r="A25" t="s">
         <v>203</v>
       </c>
@@ -6776,7 +6779,7 @@
         <v>46299</v>
       </c>
     </row>
-    <row r="26" spans="1:23">
+    <row r="26" spans="1:24">
       <c r="A26" t="s">
         <v>207</v>
       </c>
@@ -6852,7 +6855,7 @@
         <v>46299</v>
       </c>
     </row>
-    <row r="27" spans="1:23">
+    <row r="27" spans="1:24">
       <c r="A27" t="s">
         <v>212</v>
       </c>
@@ -6900,7 +6903,7 @@
         <v>0</v>
       </c>
       <c r="Q27" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R27" s="14">
         <f t="shared" si="0"/>
@@ -6912,11 +6915,11 @@
       </c>
       <c r="T27" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.4495912806539499E-3</v>
       </c>
       <c r="U27" t="str">
         <f>IF(Q27&gt;=1,"Complete",IF(Q27&gt;0,"In Progress",IF(Control!$B$7&lt;H27,"Not Started",IF(Control!$B$7&gt;I27,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V27" s="15">
         <v>46300</v>
@@ -6924,8 +6927,11 @@
       <c r="W27" s="15">
         <v>46306</v>
       </c>
-    </row>
-    <row r="28" spans="1:23">
+      <c r="X27" t="s">
+        <v>1048</v>
+      </c>
+    </row>
+    <row r="28" spans="1:24">
       <c r="A28" t="s">
         <v>218</v>
       </c>
@@ -6998,7 +7004,7 @@
         <v>46313</v>
       </c>
     </row>
-    <row r="29" spans="1:23">
+    <row r="29" spans="1:24">
       <c r="A29" t="s">
         <v>222</v>
       </c>
@@ -7071,7 +7077,7 @@
         <v>46313</v>
       </c>
     </row>
-    <row r="30" spans="1:23">
+    <row r="30" spans="1:24">
       <c r="A30" t="s">
         <v>226</v>
       </c>
@@ -7144,7 +7150,7 @@
         <v>46320</v>
       </c>
     </row>
-    <row r="31" spans="1:23">
+    <row r="31" spans="1:24">
       <c r="A31" t="s">
         <v>232</v>
       </c>
@@ -7217,7 +7223,7 @@
         <v>46327</v>
       </c>
     </row>
-    <row r="32" spans="1:23">
+    <row r="32" spans="1:24">
       <c r="A32" t="s">
         <v>236</v>
       </c>
@@ -15443,22 +15449,22 @@
       </c>
       <c r="H11" s="6">
         <f>IFERROR(SUMIF(WBS!$D$5:$D$137,A11,WBS!$T$5:$T$137)/SUMIF(WBS!$D$5:$D$137,A11,WBS!$R$5:$R$137),0)</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I11" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="J11" s="4">
         <v>3</v>
       </c>
       <c r="K11" s="4">
         <f>COUNTIFS(WBS!$D$5:$D$137,A11,WBS!$U$5:$U$137,"Complete")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L11" s="4" t="str">
         <f>IF(H11&gt;=1,"Complete",IF(H11&gt;0,"In Progress",IF(Control!$B$7&lt;D11,"Not Started",IF(Control!$B$7&gt;E11,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>In Progress</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -16969,7 +16975,7 @@
       </c>
       <c r="I4" s="6">
         <f>IF(A4=Control!$B$7,Control!$B$11,"")</f>
-        <v>0.17111716621253398</v>
+        <v>0.17656675749318793</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="42.75">

</xml_diff>

<commit_message>
docs(c1.1): record architecture acceptance (#20)
Mark the C1.1 architecture as accepted and record PR, merged-main and CI evidence.

Update the C1.1 WBS row to 100 percent completion with acceptance traceability.
</commit_message>
<xml_diff>
--- a/ESP32_S3_SQD_Project_WBS.xlsx
+++ b/ESP32_S3_SQD_Project_WBS.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive\SQD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f91d42a59b2d5e5/SQD_WBS_Backups/B4.3_WBS_Recovery_20260726_091129/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97F445B2-9959-4A2B-953A-FF2A2BEAA89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{97F445B2-9959-4A2B-953A-FF2A2BEAA89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC2B6BFE-A532-4185-87E4-86725BF234C3}"/>
   <bookViews>
     <workbookView xWindow="-14730" yWindow="-16320" windowWidth="57840" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1973" uniqueCount="1048">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1974" uniqueCount="1049">
   <si>
     <t>ESP32-S3 Solo Program Dashboard</t>
   </si>
@@ -3319,6 +3319,9 @@
   </si>
   <si>
     <t>Parthasarathy CP</t>
+  </si>
+  <si>
+    <t>Architecture: docs/phase-c/C1.1_System_Architecture.md | PR: https://github.com/CPParthasarathy/SQD/pull/19 | Main: a56bb119c16f1f61adc0c9ab7c848496d6a2b52a | CI: https://github.com/CPParthasarathy/SQD/actions/runs/30207286673 (Quality contracts and all three ESP-IDF profiles green)</t>
   </si>
 </sst>
 </file>
@@ -3834,7 +3837,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>1.9920318725099608E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -4318,14 +4321,14 @@
       </c>
       <c r="E5" s="12">
         <f>Control!B11</f>
-        <v>0.17111716621253398</v>
+        <v>0.17656675749318793</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>6</v>
       </c>
       <c r="H5" s="12">
         <f>Control!B12</f>
-        <v>0.16021798365122608</v>
+        <v>0.16566757493188003</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="30" customHeight="1"/>
@@ -4342,7 +4345,7 @@
       </c>
       <c r="E7" s="11">
         <f>Control!B14</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>9</v>
@@ -4488,11 +4491,11 @@
       </c>
       <c r="F14" s="6">
         <f>IFERROR(SUMIF(WBS!$B$5:$B$137,A14,WBS!$T$5:$T$137)/SUMIF(WBS!$B$5:$B$137,A14,WBS!$R$5:$R$137),0)</f>
-        <v>0</v>
+        <v>1.9920318725099608E-2</v>
       </c>
       <c r="G14" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1.9920318725099608E-2</v>
       </c>
       <c r="H14" s="4">
         <f>COUNTIF(WBS!$B$5:$B$137,A14)</f>
@@ -4500,7 +4503,7 @@
       </c>
       <c r="I14" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A14,WBS!$U$5:$U$137,"Complete")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J14" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A14,WBS!$U$5:$U$137,"Late")</f>
@@ -4947,7 +4950,7 @@
       </c>
       <c r="B11" s="6">
         <f>SUM(WBS!T5:T137)</f>
-        <v>0.17111716621253398</v>
+        <v>0.17656675749318793</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>69</v>
@@ -4962,7 +4965,7 @@
       </c>
       <c r="B12" s="6">
         <f>B11-B10</f>
-        <v>0.16021798365122608</v>
+        <v>0.16566757493188003</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>70</v>
@@ -4992,7 +4995,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF(WBS!U5:U137,"Complete")</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>72</v>
@@ -6119,7 +6122,7 @@
         <v>46271</v>
       </c>
     </row>
-    <row r="17" spans="1:23">
+    <row r="17" spans="1:24">
       <c r="A17" t="s">
         <v>165</v>
       </c>
@@ -6192,7 +6195,7 @@
         <v>46271</v>
       </c>
     </row>
-    <row r="18" spans="1:23">
+    <row r="18" spans="1:24">
       <c r="A18" t="s">
         <v>169</v>
       </c>
@@ -6265,7 +6268,7 @@
         <v>46271</v>
       </c>
     </row>
-    <row r="19" spans="1:23">
+    <row r="19" spans="1:24">
       <c r="A19" t="s">
         <v>175</v>
       </c>
@@ -6338,7 +6341,7 @@
         <v>46278</v>
       </c>
     </row>
-    <row r="20" spans="1:23">
+    <row r="20" spans="1:24">
       <c r="A20" t="s">
         <v>179</v>
       </c>
@@ -6411,7 +6414,7 @@
         <v>46278</v>
       </c>
     </row>
-    <row r="21" spans="1:23">
+    <row r="21" spans="1:24">
       <c r="A21" t="s">
         <v>183</v>
       </c>
@@ -6484,7 +6487,7 @@
         <v>46285</v>
       </c>
     </row>
-    <row r="22" spans="1:23">
+    <row r="22" spans="1:24">
       <c r="A22" t="s">
         <v>189</v>
       </c>
@@ -6557,7 +6560,7 @@
         <v>46292</v>
       </c>
     </row>
-    <row r="23" spans="1:23">
+    <row r="23" spans="1:24">
       <c r="A23" t="s">
         <v>193</v>
       </c>
@@ -6630,7 +6633,7 @@
         <v>46292</v>
       </c>
     </row>
-    <row r="24" spans="1:23">
+    <row r="24" spans="1:24">
       <c r="A24" t="s">
         <v>197</v>
       </c>
@@ -6703,7 +6706,7 @@
         <v>46299</v>
       </c>
     </row>
-    <row r="25" spans="1:23">
+    <row r="25" spans="1:24">
       <c r="A25" t="s">
         <v>203</v>
       </c>
@@ -6776,7 +6779,7 @@
         <v>46299</v>
       </c>
     </row>
-    <row r="26" spans="1:23">
+    <row r="26" spans="1:24">
       <c r="A26" t="s">
         <v>207</v>
       </c>
@@ -6852,7 +6855,7 @@
         <v>46299</v>
       </c>
     </row>
-    <row r="27" spans="1:23">
+    <row r="27" spans="1:24">
       <c r="A27" t="s">
         <v>212</v>
       </c>
@@ -6900,7 +6903,7 @@
         <v>0</v>
       </c>
       <c r="Q27" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R27" s="14">
         <f t="shared" si="0"/>
@@ -6912,11 +6915,11 @@
       </c>
       <c r="T27" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.4495912806539499E-3</v>
       </c>
       <c r="U27" t="str">
         <f>IF(Q27&gt;=1,"Complete",IF(Q27&gt;0,"In Progress",IF(Control!$B$7&lt;H27,"Not Started",IF(Control!$B$7&gt;I27,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V27" s="15">
         <v>46300</v>
@@ -6924,8 +6927,11 @@
       <c r="W27" s="15">
         <v>46306</v>
       </c>
-    </row>
-    <row r="28" spans="1:23">
+      <c r="X27" t="s">
+        <v>1048</v>
+      </c>
+    </row>
+    <row r="28" spans="1:24">
       <c r="A28" t="s">
         <v>218</v>
       </c>
@@ -6998,7 +7004,7 @@
         <v>46313</v>
       </c>
     </row>
-    <row r="29" spans="1:23">
+    <row r="29" spans="1:24">
       <c r="A29" t="s">
         <v>222</v>
       </c>
@@ -7071,7 +7077,7 @@
         <v>46313</v>
       </c>
     </row>
-    <row r="30" spans="1:23">
+    <row r="30" spans="1:24">
       <c r="A30" t="s">
         <v>226</v>
       </c>
@@ -7144,7 +7150,7 @@
         <v>46320</v>
       </c>
     </row>
-    <row r="31" spans="1:23">
+    <row r="31" spans="1:24">
       <c r="A31" t="s">
         <v>232</v>
       </c>
@@ -7217,7 +7223,7 @@
         <v>46327</v>
       </c>
     </row>
-    <row r="32" spans="1:23">
+    <row r="32" spans="1:24">
       <c r="A32" t="s">
         <v>236</v>
       </c>
@@ -15443,22 +15449,22 @@
       </c>
       <c r="H11" s="6">
         <f>IFERROR(SUMIF(WBS!$D$5:$D$137,A11,WBS!$T$5:$T$137)/SUMIF(WBS!$D$5:$D$137,A11,WBS!$R$5:$R$137),0)</f>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="I11" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="J11" s="4">
         <v>3</v>
       </c>
       <c r="K11" s="4">
         <f>COUNTIFS(WBS!$D$5:$D$137,A11,WBS!$U$5:$U$137,"Complete")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L11" s="4" t="str">
         <f>IF(H11&gt;=1,"Complete",IF(H11&gt;0,"In Progress",IF(Control!$B$7&lt;D11,"Not Started",IF(Control!$B$7&gt;E11,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>In Progress</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -16969,7 +16975,7 @@
       </c>
       <c r="I4" s="6">
         <f>IF(A4=Control!$B$7,Control!$B$11,"")</f>
-        <v>0.17111716621253398</v>
+        <v>0.17656675749318793</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="42.75">

</xml_diff>

<commit_message>
docs(c1.2): record component contract acceptance
</commit_message>
<xml_diff>
--- a/ESP32_S3_SQD_Project_WBS.xlsx
+++ b/ESP32_S3_SQD_Project_WBS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f91d42a59b2d5e5/SQD_WBS_Backups/B4.3_WBS_Recovery_20260726_091129/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f91d42a59b2d5e5/SQD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{97F445B2-9959-4A2B-953A-FF2A2BEAA89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC2B6BFE-A532-4185-87E4-86725BF234C3}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{97F445B2-9959-4A2B-953A-FF2A2BEAA89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3774EB4-4559-4205-8B47-D0DF71676CF7}"/>
   <bookViews>
     <workbookView xWindow="-14730" yWindow="-16320" windowWidth="57840" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1974" uniqueCount="1049">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1975" uniqueCount="1050">
   <si>
     <t>ESP32-S3 Solo Program Dashboard</t>
   </si>
@@ -3322,6 +3322,9 @@
   </si>
   <si>
     <t>Architecture: docs/phase-c/C1.1_System_Architecture.md | PR: https://github.com/CPParthasarathy/SQD/pull/19 | Main: a56bb119c16f1f61adc0c9ab7c848496d6a2b52a | CI: https://github.com/CPParthasarathy/SQD/actions/runs/30207286673 (Quality contracts and all three ESP-IDF profiles green)</t>
+  </si>
+  <si>
+    <t>Specification: docs/phase-c/C1.2_Component_Interface_and_Runtime_Contracts.md | Contract: tools/ci/c1_2_component_contract.json | PR: https://github.com/CPParthasarathy/SQD/pull/21 | Main: bad1c88dd56e584d819c612055876a298c1e9c64 | CI: https://github.com/CPParthasarathy/SQD/actions/runs/30696078035 (Quality contracts and all three ESP-IDF profiles green; post-merge verifier and 32 host tests passed)</t>
   </si>
 </sst>
 </file>
@@ -3837,7 +3840,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.9920318725099608E-2</c:v>
+                  <c:v>5.9760956175298828E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -4321,14 +4324,14 @@
       </c>
       <c r="E5" s="12">
         <f>Control!B11</f>
-        <v>0.17656675749318793</v>
+        <v>0.18746594005449582</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>6</v>
       </c>
       <c r="H5" s="12">
         <f>Control!B12</f>
-        <v>0.16566757493188003</v>
+        <v>0.17656675749318793</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="30" customHeight="1"/>
@@ -4345,7 +4348,7 @@
       </c>
       <c r="E7" s="11">
         <f>Control!B14</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>9</v>
@@ -4491,11 +4494,11 @@
       </c>
       <c r="F14" s="6">
         <f>IFERROR(SUMIF(WBS!$B$5:$B$137,A14,WBS!$T$5:$T$137)/SUMIF(WBS!$B$5:$B$137,A14,WBS!$R$5:$R$137),0)</f>
-        <v>1.9920318725099608E-2</v>
+        <v>5.9760956175298828E-2</v>
       </c>
       <c r="G14" s="6">
         <f t="shared" si="0"/>
-        <v>1.9920318725099608E-2</v>
+        <v>5.9760956175298828E-2</v>
       </c>
       <c r="H14" s="4">
         <f>COUNTIF(WBS!$B$5:$B$137,A14)</f>
@@ -4503,7 +4506,7 @@
       </c>
       <c r="I14" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A14,WBS!$U$5:$U$137,"Complete")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A14,WBS!$U$5:$U$137,"Late")</f>
@@ -4950,7 +4953,7 @@
       </c>
       <c r="B11" s="6">
         <f>SUM(WBS!T5:T137)</f>
-        <v>0.17656675749318793</v>
+        <v>0.18746594005449582</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>69</v>
@@ -4965,7 +4968,7 @@
       </c>
       <c r="B12" s="6">
         <f>B11-B10</f>
-        <v>0.16566757493188003</v>
+        <v>0.17656675749318793</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>70</v>
@@ -4995,7 +4998,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF(WBS!U5:U137,"Complete")</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>72</v>
@@ -6979,7 +6982,7 @@
         <v>0</v>
       </c>
       <c r="Q28" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R28" s="14">
         <f t="shared" si="0"/>
@@ -6991,17 +6994,20 @@
       </c>
       <c r="T28" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.08991825613079E-2</v>
       </c>
       <c r="U28" t="str">
         <f>IF(Q28&gt;=1,"Complete",IF(Q28&gt;0,"In Progress",IF(Control!$B$7&lt;H28,"Not Started",IF(Control!$B$7&gt;I28,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V28" s="15">
         <v>46300</v>
       </c>
       <c r="W28" s="15">
         <v>46313</v>
+      </c>
+      <c r="X28" t="s">
+        <v>1049</v>
       </c>
     </row>
     <row r="29" spans="1:24">
@@ -15449,18 +15455,18 @@
       </c>
       <c r="H11" s="6">
         <f>IFERROR(SUMIF(WBS!$D$5:$D$137,A11,WBS!$T$5:$T$137)/SUMIF(WBS!$D$5:$D$137,A11,WBS!$R$5:$R$137),0)</f>
-        <v>0.25</v>
+        <v>0.75000000000000011</v>
       </c>
       <c r="I11" s="6">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.75000000000000011</v>
       </c>
       <c r="J11" s="4">
         <v>3</v>
       </c>
       <c r="K11" s="4">
         <f>COUNTIFS(WBS!$D$5:$D$137,A11,WBS!$U$5:$U$137,"Complete")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L11" s="4" t="str">
         <f>IF(H11&gt;=1,"Complete",IF(H11&gt;0,"In Progress",IF(Control!$B$7&lt;D11,"Not Started",IF(Control!$B$7&gt;E11,"Late","Ready"))))</f>
@@ -16975,7 +16981,7 @@
       </c>
       <c r="I4" s="6">
         <f>IF(A4=Control!$B$7,Control!$B$11,"")</f>
-        <v>0.17656675749318793</v>
+        <v>0.18746594005449582</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="42.75">

</xml_diff>

<commit_message>
docs(c1.2): record component contract acceptance (#22)
</commit_message>
<xml_diff>
--- a/ESP32_S3_SQD_Project_WBS.xlsx
+++ b/ESP32_S3_SQD_Project_WBS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f91d42a59b2d5e5/SQD_WBS_Backups/B4.3_WBS_Recovery_20260726_091129/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f91d42a59b2d5e5/SQD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{97F445B2-9959-4A2B-953A-FF2A2BEAA89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AC2B6BFE-A532-4185-87E4-86725BF234C3}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{97F445B2-9959-4A2B-953A-FF2A2BEAA89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3774EB4-4559-4205-8B47-D0DF71676CF7}"/>
   <bookViews>
     <workbookView xWindow="-14730" yWindow="-16320" windowWidth="57840" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1974" uniqueCount="1049">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1975" uniqueCount="1050">
   <si>
     <t>ESP32-S3 Solo Program Dashboard</t>
   </si>
@@ -3322,6 +3322,9 @@
   </si>
   <si>
     <t>Architecture: docs/phase-c/C1.1_System_Architecture.md | PR: https://github.com/CPParthasarathy/SQD/pull/19 | Main: a56bb119c16f1f61adc0c9ab7c848496d6a2b52a | CI: https://github.com/CPParthasarathy/SQD/actions/runs/30207286673 (Quality contracts and all three ESP-IDF profiles green)</t>
+  </si>
+  <si>
+    <t>Specification: docs/phase-c/C1.2_Component_Interface_and_Runtime_Contracts.md | Contract: tools/ci/c1_2_component_contract.json | PR: https://github.com/CPParthasarathy/SQD/pull/21 | Main: bad1c88dd56e584d819c612055876a298c1e9c64 | CI: https://github.com/CPParthasarathy/SQD/actions/runs/30696078035 (Quality contracts and all three ESP-IDF profiles green; post-merge verifier and 32 host tests passed)</t>
   </si>
 </sst>
 </file>
@@ -3837,7 +3840,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.9920318725099608E-2</c:v>
+                  <c:v>5.9760956175298828E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -4321,14 +4324,14 @@
       </c>
       <c r="E5" s="12">
         <f>Control!B11</f>
-        <v>0.17656675749318793</v>
+        <v>0.18746594005449582</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>6</v>
       </c>
       <c r="H5" s="12">
         <f>Control!B12</f>
-        <v>0.16566757493188003</v>
+        <v>0.17656675749318793</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="30" customHeight="1"/>
@@ -4345,7 +4348,7 @@
       </c>
       <c r="E7" s="11">
         <f>Control!B14</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>9</v>
@@ -4491,11 +4494,11 @@
       </c>
       <c r="F14" s="6">
         <f>IFERROR(SUMIF(WBS!$B$5:$B$137,A14,WBS!$T$5:$T$137)/SUMIF(WBS!$B$5:$B$137,A14,WBS!$R$5:$R$137),0)</f>
-        <v>1.9920318725099608E-2</v>
+        <v>5.9760956175298828E-2</v>
       </c>
       <c r="G14" s="6">
         <f t="shared" si="0"/>
-        <v>1.9920318725099608E-2</v>
+        <v>5.9760956175298828E-2</v>
       </c>
       <c r="H14" s="4">
         <f>COUNTIF(WBS!$B$5:$B$137,A14)</f>
@@ -4503,7 +4506,7 @@
       </c>
       <c r="I14" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A14,WBS!$U$5:$U$137,"Complete")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J14" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A14,WBS!$U$5:$U$137,"Late")</f>
@@ -4950,7 +4953,7 @@
       </c>
       <c r="B11" s="6">
         <f>SUM(WBS!T5:T137)</f>
-        <v>0.17656675749318793</v>
+        <v>0.18746594005449582</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>69</v>
@@ -4965,7 +4968,7 @@
       </c>
       <c r="B12" s="6">
         <f>B11-B10</f>
-        <v>0.16566757493188003</v>
+        <v>0.17656675749318793</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>70</v>
@@ -4995,7 +4998,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF(WBS!U5:U137,"Complete")</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>72</v>
@@ -6979,7 +6982,7 @@
         <v>0</v>
       </c>
       <c r="Q28" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R28" s="14">
         <f t="shared" si="0"/>
@@ -6991,17 +6994,20 @@
       </c>
       <c r="T28" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.08991825613079E-2</v>
       </c>
       <c r="U28" t="str">
         <f>IF(Q28&gt;=1,"Complete",IF(Q28&gt;0,"In Progress",IF(Control!$B$7&lt;H28,"Not Started",IF(Control!$B$7&gt;I28,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V28" s="15">
         <v>46300</v>
       </c>
       <c r="W28" s="15">
         <v>46313</v>
+      </c>
+      <c r="X28" t="s">
+        <v>1049</v>
       </c>
     </row>
     <row r="29" spans="1:24">
@@ -15449,18 +15455,18 @@
       </c>
       <c r="H11" s="6">
         <f>IFERROR(SUMIF(WBS!$D$5:$D$137,A11,WBS!$T$5:$T$137)/SUMIF(WBS!$D$5:$D$137,A11,WBS!$R$5:$R$137),0)</f>
-        <v>0.25</v>
+        <v>0.75000000000000011</v>
       </c>
       <c r="I11" s="6">
         <f t="shared" si="0"/>
-        <v>0.25</v>
+        <v>0.75000000000000011</v>
       </c>
       <c r="J11" s="4">
         <v>3</v>
       </c>
       <c r="K11" s="4">
         <f>COUNTIFS(WBS!$D$5:$D$137,A11,WBS!$U$5:$U$137,"Complete")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L11" s="4" t="str">
         <f>IF(H11&gt;=1,"Complete",IF(H11&gt;0,"In Progress",IF(Control!$B$7&lt;D11,"Not Started",IF(Control!$B$7&gt;E11,"Late","Ready"))))</f>
@@ -16975,7 +16981,7 @@
       </c>
       <c r="I4" s="6">
         <f>IF(A4=Control!$B$7,Control!$B$11,"")</f>
-        <v>0.17656675749318793</v>
+        <v>0.18746594005449582</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="42.75">

</xml_diff>

<commit_message>
docs(wbs): record C2.1 and C2.2 completion
</commit_message>
<xml_diff>
--- a/ESP32_S3_SQD_Project_WBS.xlsx
+++ b/ESP32_S3_SQD_Project_WBS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f91d42a59b2d5e5/SQD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{97F445B2-9959-4A2B-953A-FF2A2BEAA89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7B4A80D-B986-4F5E-91F4-2A851EA0D048}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{97F445B2-9959-4A2B-953A-FF2A2BEAA89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47CDC085-51F7-4468-A5D0-052B2B32A254}"/>
   <bookViews>
     <workbookView xWindow="-14730" yWindow="-16320" windowWidth="57840" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1976" uniqueCount="1051">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1978" uniqueCount="1053">
   <si>
     <t>ESP32-S3 Solo Program Dashboard</t>
   </si>
@@ -3328,6 +3328,12 @@
   </si>
   <si>
     <t>Gate G-C accepted 2026-08-02 | Record: docs/phase-c/C1.3_Architecture_Review_and_Gate.md | PR: https://github.com/CPParthasarathy/SQD/pull/23 | Accepted main: bd995912fb5632394f6aa29b146f17ec9dcdcf6d | CI: https://github.com/CPParthasarathy/SQD/actions/runs/30745138225 (4/4 PASS) | Architecture: 11/11 PASS | C1.3 tests: 6/6 PASS | Host tests: 38/38 PASS</t>
+  </si>
+  <si>
+    <t>Document: docs/phase-c/C2.1_Board_Pins_Revision_Detection.md | Accepted main: d16f0d3223fa8d895f65837450acb346d3256b22 | Result: board-pin, active-level, pull, electrical-capability and revision-detection contract accepted, synchronized and closed</t>
+  </si>
+  <si>
+    <t>Document: docs/phase-c/C2.2_Board_Support_Implementation.md | Accepted main: 974b56aacb975b8dd719432389f34b01772eba68 | Result: static board contract PASS; 57 host tests PASS; ESP-IDF 6.0.2 isolated build PASS; GitHub Actions green; squash merge accepted, synchronized and closed</t>
   </si>
 </sst>
 </file>
@@ -3843,7 +3849,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7.9681274900398433E-2</c:v>
+                  <c:v>0.13944223107569725</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -4331,14 +4337,14 @@
       </c>
       <c r="E5" s="12">
         <f>Control!B11</f>
-        <v>0.19291553133514977</v>
+        <v>0.20926430517711161</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>6</v>
       </c>
       <c r="H5" s="12">
         <f>Control!B12</f>
-        <v>0.18201634877384187</v>
+        <v>0.19836512261580372</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="30" customHeight="1"/>
@@ -4355,7 +4361,7 @@
       </c>
       <c r="E7" s="11">
         <f>Control!B14</f>
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>9</v>
@@ -4501,11 +4507,11 @@
       </c>
       <c r="F14" s="6">
         <f>IFERROR(SUMIF(WBS!$B$5:$B$137,A14,WBS!$T$5:$T$137)/SUMIF(WBS!$B$5:$B$137,A14,WBS!$R$5:$R$137),0)</f>
-        <v>7.9681274900398433E-2</v>
+        <v>0.13944223107569725</v>
       </c>
       <c r="G14" s="6">
         <f t="shared" si="0"/>
-        <v>7.9681274900398433E-2</v>
+        <v>0.13944223107569725</v>
       </c>
       <c r="H14" s="4">
         <f>COUNTIF(WBS!$B$5:$B$137,A14)</f>
@@ -4513,7 +4519,7 @@
       </c>
       <c r="I14" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A14,WBS!$U$5:$U$137,"Complete")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J14" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A14,WBS!$U$5:$U$137,"Late")</f>
@@ -4960,7 +4966,7 @@
       </c>
       <c r="B11" s="6">
         <f>SUM(WBS!T5:T137)</f>
-        <v>0.19291553133514977</v>
+        <v>0.20926430517711161</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>69</v>
@@ -4975,7 +4981,7 @@
       </c>
       <c r="B12" s="6">
         <f>B11-B10</f>
-        <v>0.18201634877384187</v>
+        <v>0.19836512261580372</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>70</v>
@@ -5005,7 +5011,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF(WBS!U5:U137,"Complete")</f>
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>72</v>
@@ -7141,7 +7147,7 @@
         <v>0</v>
       </c>
       <c r="Q30" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R30" s="14">
         <f t="shared" si="0"/>
@@ -7153,17 +7159,20 @@
       </c>
       <c r="T30" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.4495912806539499E-3</v>
       </c>
       <c r="U30" t="str">
         <f>IF(Q30&gt;=1,"Complete",IF(Q30&gt;0,"In Progress",IF(Control!$B$7&lt;H30,"Not Started",IF(Control!$B$7&gt;I30,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V30" s="15">
         <v>46314</v>
       </c>
       <c r="W30" s="15">
         <v>46320</v>
+      </c>
+      <c r="X30" t="s">
+        <v>1051</v>
       </c>
     </row>
     <row r="31" spans="1:24">
@@ -7214,7 +7223,7 @@
         <v>0</v>
       </c>
       <c r="Q31" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R31" s="14">
         <f t="shared" si="0"/>
@@ -7226,17 +7235,20 @@
       </c>
       <c r="T31" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.08991825613079E-2</v>
       </c>
       <c r="U31" t="str">
         <f>IF(Q31&gt;=1,"Complete",IF(Q31&gt;0,"In Progress",IF(Control!$B$7&lt;H31,"Not Started",IF(Control!$B$7&gt;I31,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V31" s="15">
         <v>46314</v>
       </c>
       <c r="W31" s="15">
         <v>46327</v>
+      </c>
+      <c r="X31" t="s">
+        <v>1052</v>
       </c>
     </row>
     <row r="32" spans="1:24">
@@ -15508,22 +15520,22 @@
       </c>
       <c r="H12" s="6">
         <f>IFERROR(SUMIF(WBS!$D$5:$D$137,A12,WBS!$T$5:$T$137)/SUMIF(WBS!$D$5:$D$137,A12,WBS!$R$5:$R$137),0)</f>
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="I12" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J12" s="4">
         <v>3</v>
       </c>
       <c r="K12" s="4">
         <f>COUNTIFS(WBS!$D$5:$D$137,A12,WBS!$U$5:$U$137,"Complete")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L12" s="4" t="str">
         <f>IF(H12&gt;=1,"Complete",IF(H12&gt;0,"In Progress",IF(Control!$B$7&lt;D12,"Not Started",IF(Control!$B$7&gt;E12,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>In Progress</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -16991,7 +17003,7 @@
       </c>
       <c r="I4" s="6">
         <f>IF(A4=Control!$B$7,Control!$B$11,"")</f>
-        <v>0.19291553133514977</v>
+        <v>0.20926430517711161</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="42.75">

</xml_diff>

<commit_message>
docs(wbs): record C2.1 and C2.2 completion (#27)
</commit_message>
<xml_diff>
--- a/ESP32_S3_SQD_Project_WBS.xlsx
+++ b/ESP32_S3_SQD_Project_WBS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f91d42a59b2d5e5/SQD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{97F445B2-9959-4A2B-953A-FF2A2BEAA89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7B4A80D-B986-4F5E-91F4-2A851EA0D048}"/>
+  <xr:revisionPtr revIDLastSave="19" documentId="13_ncr:1_{97F445B2-9959-4A2B-953A-FF2A2BEAA89D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47CDC085-51F7-4468-A5D0-052B2B32A254}"/>
   <bookViews>
     <workbookView xWindow="-14730" yWindow="-16320" windowWidth="57840" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1976" uniqueCount="1051">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1978" uniqueCount="1053">
   <si>
     <t>ESP32-S3 Solo Program Dashboard</t>
   </si>
@@ -3328,6 +3328,12 @@
   </si>
   <si>
     <t>Gate G-C accepted 2026-08-02 | Record: docs/phase-c/C1.3_Architecture_Review_and_Gate.md | PR: https://github.com/CPParthasarathy/SQD/pull/23 | Accepted main: bd995912fb5632394f6aa29b146f17ec9dcdcf6d | CI: https://github.com/CPParthasarathy/SQD/actions/runs/30745138225 (4/4 PASS) | Architecture: 11/11 PASS | C1.3 tests: 6/6 PASS | Host tests: 38/38 PASS</t>
+  </si>
+  <si>
+    <t>Document: docs/phase-c/C2.1_Board_Pins_Revision_Detection.md | Accepted main: d16f0d3223fa8d895f65837450acb346d3256b22 | Result: board-pin, active-level, pull, electrical-capability and revision-detection contract accepted, synchronized and closed</t>
+  </si>
+  <si>
+    <t>Document: docs/phase-c/C2.2_Board_Support_Implementation.md | Accepted main: 974b56aacb975b8dd719432389f34b01772eba68 | Result: static board contract PASS; 57 host tests PASS; ESP-IDF 6.0.2 isolated build PASS; GitHub Actions green; squash merge accepted, synchronized and closed</t>
   </si>
 </sst>
 </file>
@@ -3843,7 +3849,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7.9681274900398433E-2</c:v>
+                  <c:v>0.13944223107569725</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -4331,14 +4337,14 @@
       </c>
       <c r="E5" s="12">
         <f>Control!B11</f>
-        <v>0.19291553133514977</v>
+        <v>0.20926430517711161</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>6</v>
       </c>
       <c r="H5" s="12">
         <f>Control!B12</f>
-        <v>0.18201634877384187</v>
+        <v>0.19836512261580372</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="30" customHeight="1"/>
@@ -4355,7 +4361,7 @@
       </c>
       <c r="E7" s="11">
         <f>Control!B14</f>
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>9</v>
@@ -4501,11 +4507,11 @@
       </c>
       <c r="F14" s="6">
         <f>IFERROR(SUMIF(WBS!$B$5:$B$137,A14,WBS!$T$5:$T$137)/SUMIF(WBS!$B$5:$B$137,A14,WBS!$R$5:$R$137),0)</f>
-        <v>7.9681274900398433E-2</v>
+        <v>0.13944223107569725</v>
       </c>
       <c r="G14" s="6">
         <f t="shared" si="0"/>
-        <v>7.9681274900398433E-2</v>
+        <v>0.13944223107569725</v>
       </c>
       <c r="H14" s="4">
         <f>COUNTIF(WBS!$B$5:$B$137,A14)</f>
@@ -4513,7 +4519,7 @@
       </c>
       <c r="I14" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A14,WBS!$U$5:$U$137,"Complete")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J14" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A14,WBS!$U$5:$U$137,"Late")</f>
@@ -4960,7 +4966,7 @@
       </c>
       <c r="B11" s="6">
         <f>SUM(WBS!T5:T137)</f>
-        <v>0.19291553133514977</v>
+        <v>0.20926430517711161</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>69</v>
@@ -4975,7 +4981,7 @@
       </c>
       <c r="B12" s="6">
         <f>B11-B10</f>
-        <v>0.18201634877384187</v>
+        <v>0.19836512261580372</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>70</v>
@@ -5005,7 +5011,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF(WBS!U5:U137,"Complete")</f>
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>72</v>
@@ -7141,7 +7147,7 @@
         <v>0</v>
       </c>
       <c r="Q30" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R30" s="14">
         <f t="shared" si="0"/>
@@ -7153,17 +7159,20 @@
       </c>
       <c r="T30" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.4495912806539499E-3</v>
       </c>
       <c r="U30" t="str">
         <f>IF(Q30&gt;=1,"Complete",IF(Q30&gt;0,"In Progress",IF(Control!$B$7&lt;H30,"Not Started",IF(Control!$B$7&gt;I30,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V30" s="15">
         <v>46314</v>
       </c>
       <c r="W30" s="15">
         <v>46320</v>
+      </c>
+      <c r="X30" t="s">
+        <v>1051</v>
       </c>
     </row>
     <row r="31" spans="1:24">
@@ -7214,7 +7223,7 @@
         <v>0</v>
       </c>
       <c r="Q31" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R31" s="14">
         <f t="shared" si="0"/>
@@ -7226,17 +7235,20 @@
       </c>
       <c r="T31" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.08991825613079E-2</v>
       </c>
       <c r="U31" t="str">
         <f>IF(Q31&gt;=1,"Complete",IF(Q31&gt;0,"In Progress",IF(Control!$B$7&lt;H31,"Not Started",IF(Control!$B$7&gt;I31,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V31" s="15">
         <v>46314</v>
       </c>
       <c r="W31" s="15">
         <v>46327</v>
+      </c>
+      <c r="X31" t="s">
+        <v>1052</v>
       </c>
     </row>
     <row r="32" spans="1:24">
@@ -15508,22 +15520,22 @@
       </c>
       <c r="H12" s="6">
         <f>IFERROR(SUMIF(WBS!$D$5:$D$137,A12,WBS!$T$5:$T$137)/SUMIF(WBS!$D$5:$D$137,A12,WBS!$R$5:$R$137),0)</f>
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="I12" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="J12" s="4">
         <v>3</v>
       </c>
       <c r="K12" s="4">
         <f>COUNTIFS(WBS!$D$5:$D$137,A12,WBS!$U$5:$U$137,"Complete")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L12" s="4" t="str">
         <f>IF(H12&gt;=1,"Complete",IF(H12&gt;0,"In Progress",IF(Control!$B$7&lt;D12,"Not Started",IF(Control!$B$7&gt;E12,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>In Progress</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -16991,7 +17003,7 @@
       </c>
       <c r="I4" s="6">
         <f>IF(A4=Control!$B$7,Control!$B$11,"")</f>
-        <v>0.19291553133514977</v>
+        <v>0.20926430517711161</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="42.75">

</xml_diff>